<commit_message>
Achieved higher accruacy rates with 10. Will need to check out on applicability here too
</commit_message>
<xml_diff>
--- a/LLM_Extraction_and_CrossCritique/interactive-table/SQL_Results_Cat3_Working_Query.xlsx
+++ b/LLM_Extraction_and_CrossCritique/interactive-table/SQL_Results_Cat3_Working_Query.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhrub\Mayo-CoRAL\LLM_Extraction_and_CrossCritique\interactive-table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E580F064-C127-4B94-819C-F40A0A65F1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF441875-3AA7-46A1-B7DD-582F1E028689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1812" yWindow="1812" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -4424,7 +4424,7 @@
     <col min="7" max="7" width="61" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4444,7 +4444,10 @@
         <v>975</v>
       </c>
     </row>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
@@ -4464,7 +4467,10 @@
         <v>977</v>
       </c>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
@@ -4484,7 +4490,10 @@
         <v>979</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
@@ -4504,7 +4513,10 @@
         <v>981</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
@@ -4524,7 +4536,10 @@
         <v>983</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
       <c r="B6" t="s">
         <v>13</v>
       </c>
@@ -4544,7 +4559,10 @@
         <v>985</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
       <c r="B7" t="s">
         <v>15</v>
       </c>
@@ -4564,7 +4582,10 @@
         <v>987</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
       <c r="B8" t="s">
         <v>17</v>
       </c>
@@ -4584,7 +4605,10 @@
         <v>989</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
       <c r="B9" t="s">
         <v>19</v>
       </c>
@@ -4604,7 +4628,10 @@
         <v>990</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
       <c r="B10" t="s">
         <v>21</v>
       </c>
@@ -4624,7 +4651,10 @@
         <v>992</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
       <c r="B11" t="s">
         <v>23</v>
       </c>
@@ -4644,7 +4674,10 @@
         <v>983</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
       <c r="B12" t="s">
         <v>25</v>
       </c>
@@ -4664,7 +4697,10 @@
         <v>987</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
       <c r="B13" t="s">
         <v>27</v>
       </c>
@@ -4684,7 +4720,10 @@
         <v>994</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
       <c r="B14" t="s">
         <v>29</v>
       </c>
@@ -4704,7 +4743,10 @@
         <v>983</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
       <c r="B15" t="s">
         <v>31</v>
       </c>
@@ -4724,7 +4766,10 @@
         <v>995</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
       <c r="B16" t="s">
         <v>33</v>
       </c>
@@ -4744,7 +4789,10 @@
         <v>997</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
       <c r="B17" t="s">
         <v>35</v>
       </c>
@@ -4764,7 +4812,10 @@
         <v>983</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
       <c r="B18" t="s">
         <v>37</v>
       </c>
@@ -4784,7 +4835,10 @@
         <v>999</v>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
       <c r="B19" t="s">
         <v>39</v>
       </c>
@@ -4804,7 +4858,10 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
       <c r="B20" t="s">
         <v>41</v>
       </c>
@@ -4824,7 +4881,10 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
       <c r="B21" t="s">
         <v>43</v>
       </c>
@@ -4844,7 +4904,10 @@
         <v>983</v>
       </c>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>21</v>
+      </c>
       <c r="B22" t="s">
         <v>45</v>
       </c>
@@ -4864,7 +4927,10 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>22</v>
+      </c>
       <c r="B23" t="s">
         <v>47</v>
       </c>
@@ -4884,7 +4950,10 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>23</v>
+      </c>
       <c r="B24" t="s">
         <v>49</v>
       </c>
@@ -4904,7 +4973,10 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>24</v>
+      </c>
       <c r="B25" t="s">
         <v>51</v>
       </c>
@@ -4924,7 +4996,10 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>25</v>
+      </c>
       <c r="B26" t="s">
         <v>53</v>
       </c>
@@ -4944,7 +5019,10 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>26</v>
+      </c>
       <c r="B27" t="s">
         <v>55</v>
       </c>
@@ -4964,7 +5042,10 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>27</v>
+      </c>
       <c r="B28" t="s">
         <v>57</v>
       </c>
@@ -4984,7 +5065,10 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>28</v>
+      </c>
       <c r="B29" t="s">
         <v>59</v>
       </c>
@@ -5004,7 +5088,10 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>29</v>
+      </c>
       <c r="B30" t="s">
         <v>61</v>
       </c>
@@ -5024,7 +5111,10 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>30</v>
+      </c>
       <c r="B31" t="s">
         <v>63</v>
       </c>
@@ -5044,7 +5134,10 @@
         <v>985</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
       <c r="B32" t="s">
         <v>65</v>
       </c>
@@ -5064,7 +5157,10 @@
         <v>994</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>32</v>
+      </c>
       <c r="B33" t="s">
         <v>67</v>
       </c>
@@ -5084,7 +5180,10 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>33</v>
+      </c>
       <c r="B34" t="s">
         <v>69</v>
       </c>
@@ -5104,7 +5203,10 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>34</v>
+      </c>
       <c r="B35" t="s">
         <v>71</v>
       </c>
@@ -5124,7 +5226,10 @@
         <v>981</v>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>35</v>
+      </c>
       <c r="B36" t="s">
         <v>73</v>
       </c>
@@ -5144,7 +5249,10 @@
         <v>977</v>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>36</v>
+      </c>
       <c r="B37" t="s">
         <v>75</v>
       </c>
@@ -5164,7 +5272,10 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>37</v>
+      </c>
       <c r="B38" t="s">
         <v>77</v>
       </c>
@@ -5184,7 +5295,10 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>38</v>
+      </c>
       <c r="B39" t="s">
         <v>79</v>
       </c>
@@ -5204,7 +5318,10 @@
         <v>987</v>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>39</v>
+      </c>
       <c r="B40" t="s">
         <v>81</v>
       </c>
@@ -5224,7 +5341,10 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>40</v>
+      </c>
       <c r="B41" t="s">
         <v>83</v>
       </c>
@@ -5244,7 +5364,10 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>41</v>
+      </c>
       <c r="B42" t="s">
         <v>85</v>
       </c>
@@ -5264,7 +5387,10 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>42</v>
+      </c>
       <c r="B43" t="s">
         <v>87</v>
       </c>
@@ -5284,7 +5410,10 @@
         <v>995</v>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>43</v>
+      </c>
       <c r="B44" t="s">
         <v>89</v>
       </c>
@@ -5304,7 +5433,10 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>44</v>
+      </c>
       <c r="B45" t="s">
         <v>91</v>
       </c>
@@ -5324,7 +5456,10 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>45</v>
+      </c>
       <c r="B46" t="s">
         <v>93</v>
       </c>
@@ -5344,7 +5479,10 @@
         <v>985</v>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>46</v>
+      </c>
       <c r="B47" t="s">
         <v>95</v>
       </c>
@@ -5364,7 +5502,10 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>47</v>
+      </c>
       <c r="B48" t="s">
         <v>97</v>
       </c>
@@ -5384,7 +5525,10 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>48</v>
+      </c>
       <c r="B49" t="s">
         <v>99</v>
       </c>
@@ -5404,7 +5548,10 @@
         <v>987</v>
       </c>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>49</v>
+      </c>
       <c r="B50" t="s">
         <v>101</v>
       </c>
@@ -5424,7 +5571,10 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>50</v>
+      </c>
       <c r="B51" t="s">
         <v>103</v>
       </c>
@@ -5444,7 +5594,10 @@
         <v>979</v>
       </c>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>51</v>
+      </c>
       <c r="B52" t="s">
         <v>105</v>
       </c>
@@ -5464,7 +5617,10 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>52</v>
+      </c>
       <c r="B53" t="s">
         <v>107</v>
       </c>
@@ -5484,7 +5640,10 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>53</v>
+      </c>
       <c r="B54" t="s">
         <v>109</v>
       </c>
@@ -5504,7 +5663,10 @@
         <v>995</v>
       </c>
     </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>54</v>
+      </c>
       <c r="B55" t="s">
         <v>111</v>
       </c>
@@ -5524,7 +5686,10 @@
         <v>987</v>
       </c>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>55</v>
+      </c>
       <c r="B56" t="s">
         <v>113</v>
       </c>
@@ -5544,7 +5709,10 @@
         <v>997</v>
       </c>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>56</v>
+      </c>
       <c r="B57" t="s">
         <v>115</v>
       </c>
@@ -5564,7 +5732,10 @@
         <v>989</v>
       </c>
     </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>57</v>
+      </c>
       <c r="B58" t="s">
         <v>117</v>
       </c>
@@ -5584,7 +5755,10 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>58</v>
+      </c>
       <c r="B59" t="s">
         <v>119</v>
       </c>
@@ -5604,7 +5778,10 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>59</v>
+      </c>
       <c r="B60" t="s">
         <v>121</v>
       </c>
@@ -5624,7 +5801,10 @@
         <v>981</v>
       </c>
     </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>60</v>
+      </c>
       <c r="B61" t="s">
         <v>123</v>
       </c>
@@ -5644,7 +5824,10 @@
         <v>987</v>
       </c>
     </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>61</v>
+      </c>
       <c r="B62" t="s">
         <v>125</v>
       </c>
@@ -5664,7 +5847,10 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>62</v>
+      </c>
       <c r="B63" t="s">
         <v>127</v>
       </c>
@@ -5684,7 +5870,10 @@
         <v>992</v>
       </c>
     </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <v>63</v>
+      </c>
       <c r="B64" t="s">
         <v>129</v>
       </c>
@@ -5704,7 +5893,10 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>64</v>
+      </c>
       <c r="B65" t="s">
         <v>131</v>
       </c>
@@ -5724,7 +5916,10 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>65</v>
+      </c>
       <c r="B66" t="s">
         <v>133</v>
       </c>
@@ -5744,7 +5939,10 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>66</v>
+      </c>
       <c r="B67" t="s">
         <v>135</v>
       </c>
@@ -5764,7 +5962,10 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>67</v>
+      </c>
       <c r="B68" t="s">
         <v>137</v>
       </c>
@@ -5784,7 +5985,10 @@
         <v>979</v>
       </c>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>68</v>
+      </c>
       <c r="B69" t="s">
         <v>139</v>
       </c>
@@ -5804,7 +6008,10 @@
         <v>985</v>
       </c>
     </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>69</v>
+      </c>
       <c r="B70" t="s">
         <v>141</v>
       </c>
@@ -5824,7 +6031,10 @@
         <v>997</v>
       </c>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>70</v>
+      </c>
       <c r="B71" t="s">
         <v>143</v>
       </c>
@@ -5844,7 +6054,10 @@
         <v>977</v>
       </c>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>71</v>
+      </c>
       <c r="B72" t="s">
         <v>145</v>
       </c>
@@ -5864,7 +6077,10 @@
         <v>983</v>
       </c>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>72</v>
+      </c>
       <c r="B73" t="s">
         <v>147</v>
       </c>
@@ -5884,7 +6100,10 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>73</v>
+      </c>
       <c r="B74" t="s">
         <v>149</v>
       </c>
@@ -5904,7 +6123,10 @@
         <v>985</v>
       </c>
     </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>74</v>
+      </c>
       <c r="B75" t="s">
         <v>151</v>
       </c>
@@ -5924,7 +6146,10 @@
         <v>979</v>
       </c>
     </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>75</v>
+      </c>
       <c r="B76" t="s">
         <v>153</v>
       </c>
@@ -5944,7 +6169,10 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>76</v>
+      </c>
       <c r="B77" t="s">
         <v>155</v>
       </c>
@@ -5964,7 +6192,10 @@
         <v>995</v>
       </c>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>77</v>
+      </c>
       <c r="B78" t="s">
         <v>157</v>
       </c>
@@ -5984,7 +6215,10 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>78</v>
+      </c>
       <c r="B79" t="s">
         <v>159</v>
       </c>
@@ -6004,7 +6238,10 @@
         <v>997</v>
       </c>
     </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>79</v>
+      </c>
       <c r="B80" t="s">
         <v>161</v>
       </c>
@@ -6024,7 +6261,10 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>80</v>
+      </c>
       <c r="B81" t="s">
         <v>163</v>
       </c>
@@ -6044,7 +6284,10 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>81</v>
+      </c>
       <c r="B82" t="s">
         <v>165</v>
       </c>
@@ -6064,7 +6307,10 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>82</v>
+      </c>
       <c r="B83" t="s">
         <v>167</v>
       </c>
@@ -6084,7 +6330,10 @@
         <v>977</v>
       </c>
     </row>
-    <row r="84" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>83</v>
+      </c>
       <c r="B84" t="s">
         <v>169</v>
       </c>
@@ -6104,7 +6353,10 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>84</v>
+      </c>
       <c r="B85" t="s">
         <v>171</v>
       </c>
@@ -6124,7 +6376,10 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>85</v>
+      </c>
       <c r="B86" t="s">
         <v>173</v>
       </c>
@@ -6144,7 +6399,10 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>86</v>
+      </c>
       <c r="B87" t="s">
         <v>175</v>
       </c>
@@ -6164,7 +6422,10 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>87</v>
+      </c>
       <c r="B88" t="s">
         <v>177</v>
       </c>
@@ -6184,7 +6445,10 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>88</v>
+      </c>
       <c r="B89" t="s">
         <v>179</v>
       </c>
@@ -6204,7 +6468,10 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>89</v>
+      </c>
       <c r="B90" t="s">
         <v>181</v>
       </c>
@@ -6224,7 +6491,10 @@
         <v>995</v>
       </c>
     </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>90</v>
+      </c>
       <c r="B91" t="s">
         <v>183</v>
       </c>
@@ -6244,7 +6514,10 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>91</v>
+      </c>
       <c r="B92" t="s">
         <v>185</v>
       </c>
@@ -6264,7 +6537,10 @@
         <v>979</v>
       </c>
     </row>
-    <row r="93" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>92</v>
+      </c>
       <c r="B93" t="s">
         <v>187</v>
       </c>
@@ -6284,7 +6560,10 @@
         <v>981</v>
       </c>
     </row>
-    <row r="94" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>93</v>
+      </c>
       <c r="B94" t="s">
         <v>189</v>
       </c>
@@ -6304,7 +6583,10 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A95">
+        <v>94</v>
+      </c>
       <c r="B95" t="s">
         <v>191</v>
       </c>
@@ -6324,7 +6606,10 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96">
+        <v>95</v>
+      </c>
       <c r="B96" t="s">
         <v>193</v>
       </c>
@@ -6345,6 +6630,9 @@
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97">
+        <v>96</v>
+      </c>
       <c r="B97" t="s">
         <v>195</v>
       </c>
@@ -6365,6 +6653,9 @@
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98">
+        <v>97</v>
+      </c>
       <c r="B98" t="s">
         <v>197</v>
       </c>
@@ -6385,6 +6676,9 @@
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99">
+        <v>98</v>
+      </c>
       <c r="B99" t="s">
         <v>199</v>
       </c>
@@ -6405,6 +6699,9 @@
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100">
+        <v>99</v>
+      </c>
       <c r="B100" t="s">
         <v>201</v>
       </c>
@@ -6425,6 +6722,9 @@
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101">
+        <v>100</v>
+      </c>
       <c r="B101" t="s">
         <v>203</v>
       </c>

</xml_diff>